<commit_message>
Reflect WasteWerx guidance on staffing (worst-case + cross-training)
Per Vincent Tizio (WasteWerx, 5/27/26 email via Glen): the 62-FTE staffing pro
forma is intentional worst-case 'overkill'; cross-trained roles reduce headcount;
health-insurance/benefits need actuals; salaries are FL market pending Robert's
Michigan adjustment.

Adds an editable cross-training/efficiency factor (xtrain, default 1.0 = worst
case) alongside the Michigan labor adjustment (mi_adj). Labor now flexes:
labor_fl x mi_adj x xtrain. Notes/caveats updated to cite the source and flag that
net labor could move down (cross-training) or up (MI rates + real benefits). Zero
formula errors; worst-case default leaves prior figures unchanged.

https://claude.ai/code/session_01NNVRfcBeiW4jRftzrwemzW
</commit_message>
<xml_diff>
--- a/docs/business/MichiganLTC_Network_Financial_Model_FINAL.xlsx
+++ b/docs/business/MichiganLTC_Network_Financial_Model_FINAL.xlsx
@@ -82,12 +82,12 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00E2EFDA"/>
+        <fgColor rgb="00FCE4D6"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FCE4D6"/>
+        <fgColor rgb="00E2EFDA"/>
       </patternFill>
     </fill>
   </fills>
@@ -135,21 +135,21 @@
     <xf numFmtId="3" fontId="0" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="3" fontId="0" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="3" fontId="6" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="3" fontId="6" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="3" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="3" fontId="6" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="3" fontId="6" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="3" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="3" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="3" fontId="6" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="3" fontId="6" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="3" fontId="6" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="3" fontId="0" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="3" fontId="0" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="3" fontId="6" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
@@ -686,7 +686,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E36"/>
+  <dimension ref="A1:E37"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1083,48 +1083,48 @@
       </c>
       <c r="E18" s="2" t="inlineStr">
         <is>
-          <t>FL-&gt;MI cost-of-living [CONFIRM]</t>
+          <t>FL-&gt;MI cost-of-living [Robert to set]</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="5" t="inlineStr">
         <is>
-          <t>feedstock</t>
+          <t>xtrain</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Net feedstock cost (negative if tipping-fee positive)</t>
-        </is>
-      </c>
-      <c r="C19" s="6" t="n">
-        <v>0</v>
+          <t>Cross-training / headcount efficiency factor</t>
+        </is>
+      </c>
+      <c r="C19" s="7" t="n">
+        <v>1</v>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>$/yr</t>
+          <t>x</t>
         </is>
       </c>
       <c r="E19" s="2" t="inlineStr">
         <is>
-          <t>[CONFIRM — tires may carry tipping fees]</t>
+          <t>WasteWerx (V.Tizio 5/27): staffing is WORST-CASE; cross-training reduces it [set &lt;1.0]</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="5" t="inlineStr">
         <is>
-          <t>utilities</t>
+          <t>feedstock</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Utilities / energy (net of syngas self-supply)</t>
-        </is>
-      </c>
-      <c r="C20" s="8" t="n">
-        <v>1200000</v>
+          <t>Net feedstock cost (negative if tipping-fee positive)</t>
+        </is>
+      </c>
+      <c r="C20" s="6" t="n">
+        <v>0</v>
       </c>
       <c r="D20" t="inlineStr">
         <is>
@@ -1133,23 +1133,23 @@
       </c>
       <c r="E20" s="2" t="inlineStr">
         <is>
-          <t>ESTIMATE [CONFIRM]</t>
+          <t>[CONFIRM — tires may carry tipping fees]</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="5" t="inlineStr">
         <is>
-          <t>maint</t>
+          <t>utilities</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Maintenance materials + contract maintenance</t>
+          <t>Utilities / energy (net of syngas self-supply)</t>
         </is>
       </c>
       <c r="C21" s="8" t="n">
-        <v>500000</v>
+        <v>1200000</v>
       </c>
       <c r="D21" t="inlineStr">
         <is>
@@ -1165,16 +1165,16 @@
     <row r="22">
       <c r="A22" s="5" t="inlineStr">
         <is>
-          <t>insurance</t>
+          <t>maint</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Insurance (industrial)</t>
+          <t>Maintenance materials + contract maintenance</t>
         </is>
       </c>
       <c r="C22" s="8" t="n">
-        <v>400000</v>
+        <v>500000</v>
       </c>
       <c r="D22" t="inlineStr">
         <is>
@@ -1190,16 +1190,16 @@
     <row r="23">
       <c r="A23" s="5" t="inlineStr">
         <is>
-          <t>contracted</t>
+          <t>insurance</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Contracted svcs (security/janitorial/IT/3rd-party MRV verification)</t>
+          <t>Insurance (industrial)</t>
         </is>
       </c>
       <c r="C23" s="8" t="n">
-        <v>350000</v>
+        <v>400000</v>
       </c>
       <c r="D23" t="inlineStr">
         <is>
@@ -1208,23 +1208,23 @@
       </c>
       <c r="E23" s="2" t="inlineStr">
         <is>
-          <t>NOT in staffing pro forma — budget separately [CONFIRM]</t>
+          <t>ESTIMATE [CONFIRM]</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="5" t="inlineStr">
         <is>
-          <t>ga</t>
+          <t>contracted</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>G&amp;A / SG&amp;A (corporate alloc, legal, accounting, software)</t>
+          <t>Contracted svcs (security/janitorial/IT/3rd-party MRV verification)</t>
         </is>
       </c>
       <c r="C24" s="8" t="n">
-        <v>750000</v>
+        <v>350000</v>
       </c>
       <c r="D24" t="inlineStr">
         <is>
@@ -1233,48 +1233,48 @@
       </c>
       <c r="E24" s="2" t="inlineStr">
         <is>
-          <t>ESTIMATE [CONFIRM]</t>
+          <t>NOT in staffing pro forma — budget separately [CONFIRM]</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="5" t="inlineStr">
         <is>
-          <t>raise_site</t>
+          <t>ga</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Project raise per site</t>
+          <t>G&amp;A / SG&amp;A (corporate alloc, legal, accounting, software)</t>
         </is>
       </c>
       <c r="C25" s="8" t="n">
-        <v>15000000</v>
+        <v>750000</v>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>$</t>
+          <t>$/yr</t>
         </is>
       </c>
       <c r="E25" s="2" t="inlineStr">
         <is>
-          <t>sponsor-directed headline</t>
+          <t>ESTIMATE [CONFIRM]</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="5" t="inlineStr">
         <is>
-          <t>build</t>
+          <t>raise_site</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Use of funds: build / core plant</t>
+          <t>Project raise per site</t>
         </is>
       </c>
       <c r="C26" s="8" t="n">
-        <v>8000000</v>
+        <v>15000000</v>
       </c>
       <c r="D26" t="inlineStr">
         <is>
@@ -1283,23 +1283,23 @@
       </c>
       <c r="E26" s="2" t="inlineStr">
         <is>
-          <t>rough verbal</t>
+          <t>sponsor-directed headline</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="5" t="inlineStr">
         <is>
-          <t>addl</t>
+          <t>build</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Use of funds: added construction</t>
+          <t>Use of funds: build / core plant</t>
         </is>
       </c>
       <c r="C27" s="8" t="n">
-        <v>1000000</v>
+        <v>8000000</v>
       </c>
       <c r="D27" t="inlineStr">
         <is>
@@ -1315,16 +1315,16 @@
     <row r="28">
       <c r="A28" s="5" t="inlineStr">
         <is>
-          <t>preproc</t>
+          <t>addl</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Use of funds: pre-processing/pre-treatment equip</t>
+          <t>Use of funds: added construction</t>
         </is>
       </c>
       <c r="C28" s="8" t="n">
-        <v>2000000</v>
+        <v>1000000</v>
       </c>
       <c r="D28" t="inlineStr">
         <is>
@@ -1340,16 +1340,16 @@
     <row r="29">
       <c r="A29" s="5" t="inlineStr">
         <is>
-          <t>conting</t>
+          <t>preproc</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>Use of funds: contingency/fees/payroll/training</t>
+          <t>Use of funds: pre-processing/pre-treatment equip</t>
         </is>
       </c>
       <c r="C29" s="8" t="n">
-        <v>5000000</v>
+        <v>2000000</v>
       </c>
       <c r="D29" t="inlineStr">
         <is>
@@ -1365,16 +1365,16 @@
     <row r="30">
       <c r="A30" s="5" t="inlineStr">
         <is>
-          <t>ww_license</t>
+          <t>conting</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>WasteWerx license fee (Yr1, net of design credit)</t>
+          <t>Use of funds: contingency/fees/payroll/training</t>
         </is>
       </c>
       <c r="C30" s="8" t="n">
-        <v>5450000</v>
+        <v>5000000</v>
       </c>
       <c r="D30" t="inlineStr">
         <is>
@@ -1383,23 +1383,23 @@
       </c>
       <c r="E30" s="2" t="inlineStr">
         <is>
-          <t>signed Model 3</t>
+          <t>rough verbal</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="5" t="inlineStr">
         <is>
-          <t>ww_design</t>
+          <t>ww_license</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>WasteWerx design fee (credited)</t>
+          <t>WasteWerx license fee (Yr1, net of design credit)</t>
         </is>
       </c>
       <c r="C31" s="8" t="n">
-        <v>50000</v>
+        <v>5450000</v>
       </c>
       <c r="D31" t="inlineStr">
         <is>
@@ -1415,16 +1415,16 @@
     <row r="32">
       <c r="A32" s="5" t="inlineStr">
         <is>
-          <t>ww_monitor</t>
+          <t>ww_design</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>WasteWerx Yr1 monitoring fees</t>
+          <t>WasteWerx design fee (credited)</t>
         </is>
       </c>
       <c r="C32" s="8" t="n">
-        <v>175000</v>
+        <v>50000</v>
       </c>
       <c r="D32" t="inlineStr">
         <is>
@@ -1440,16 +1440,16 @@
     <row r="33">
       <c r="A33" s="5" t="inlineStr">
         <is>
-          <t>ww_royalty</t>
+          <t>ww_monitor</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>WasteWerx Yr1 production royalty</t>
+          <t>WasteWerx Yr1 monitoring fees</t>
         </is>
       </c>
       <c r="C33" s="8" t="n">
-        <v>995328</v>
+        <v>175000</v>
       </c>
       <c r="D33" t="inlineStr">
         <is>
@@ -1465,16 +1465,16 @@
     <row r="34">
       <c r="A34" s="5" t="inlineStr">
         <is>
-          <t>cust_capex</t>
+          <t>ww_royalty</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>Customer-side capex (site/utilities/permits/WC)</t>
+          <t>WasteWerx Yr1 production royalty</t>
         </is>
       </c>
       <c r="C34" s="8" t="n">
-        <v>952500</v>
+        <v>995328</v>
       </c>
       <c r="D34" t="inlineStr">
         <is>
@@ -1490,16 +1490,16 @@
     <row r="35">
       <c r="A35" s="5" t="inlineStr">
         <is>
-          <t>company_raise</t>
+          <t>cust_capex</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>Company-level raise (separate)</t>
+          <t>Customer-side capex (site/utilities/permits/WC)</t>
         </is>
       </c>
       <c r="C35" s="8" t="n">
-        <v>2500000</v>
+        <v>952500</v>
       </c>
       <c r="D35" t="inlineStr">
         <is>
@@ -1508,30 +1508,55 @@
       </c>
       <c r="E35" s="2" t="inlineStr">
         <is>
-          <t>sponsor-directed</t>
+          <t>signed Model 3</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="5" t="inlineStr">
         <is>
+          <t>company_raise</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>Company-level raise (separate)</t>
+        </is>
+      </c>
+      <c r="C36" s="8" t="n">
+        <v>2500000</v>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>$</t>
+        </is>
+      </c>
+      <c r="E36" s="2" t="inlineStr">
+        <is>
+          <t>sponsor-directed</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="5" t="inlineStr">
+        <is>
           <t>sites</t>
         </is>
       </c>
-      <c r="B36" t="inlineStr">
+      <c r="B37" t="inlineStr">
         <is>
           <t>Number of sites in network</t>
         </is>
       </c>
-      <c r="C36" s="6" t="n">
+      <c r="C37" s="6" t="n">
         <v>3</v>
       </c>
-      <c r="D36" t="inlineStr">
+      <c r="D37" t="inlineStr">
         <is>
           <t>#</t>
         </is>
       </c>
-      <c r="E36" s="2" t="inlineStr">
+      <c r="E37" s="2" t="inlineStr">
         <is>
           <t>Michigan corridor</t>
         </is>
@@ -1548,7 +1573,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C20"/>
+  <dimension ref="A1:C23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="54" customWidth="1" min="1" max="1"/>
@@ -1590,16 +1615,16 @@
     <row r="5">
       <c r="A5" s="9" t="inlineStr">
         <is>
-          <t>Site labor — loaded, 62 FTE (MI-adjusted)</t>
+          <t>Site labor — loaded (62 FTE worst-case x MI-adj x cross-training)</t>
         </is>
       </c>
       <c r="B5" s="10">
-        <f>Inputs!$C$17*Inputs!$C$18</f>
+        <f>Inputs!$C$17*Inputs!$C$18*Inputs!$C$19</f>
         <v/>
       </c>
       <c r="C5" s="9" t="inlineStr">
         <is>
-          <t>KNOWN — WasteWerx staffing pro forma</t>
+          <t>WORST-CASE per WasteWerx (V.Tizio); benefits/MI rates need actuals [Robert]</t>
         </is>
       </c>
     </row>
@@ -1609,8 +1634,8 @@
           <t>WasteWerx production royalty (recurring)</t>
         </is>
       </c>
-      <c r="B6" s="10">
-        <f>Inputs!$C$33</f>
+      <c r="B6" s="11">
+        <f>Inputs!$C$34</f>
         <v/>
       </c>
       <c r="C6" s="9" t="inlineStr">
@@ -1625,8 +1650,8 @@
           <t>WasteWerx monitoring fees (recurring)</t>
         </is>
       </c>
-      <c r="B7" s="10">
-        <f>Inputs!$C$32</f>
+      <c r="B7" s="11">
+        <f>Inputs!$C$33</f>
         <v/>
       </c>
       <c r="C7" s="9" t="inlineStr">
@@ -1641,8 +1666,8 @@
           <t>Net feedstock cost</t>
         </is>
       </c>
-      <c r="B8" s="11">
-        <f>Inputs!$C$19</f>
+      <c r="B8" s="10">
+        <f>Inputs!$C$20</f>
         <v/>
       </c>
       <c r="C8" s="9" t="inlineStr">
@@ -1657,8 +1682,8 @@
           <t>Utilities / energy (net of syngas self-supply)</t>
         </is>
       </c>
-      <c r="B9" s="11">
-        <f>Inputs!$C$20</f>
+      <c r="B9" s="10">
+        <f>Inputs!$C$21</f>
         <v/>
       </c>
       <c r="C9" s="9" t="inlineStr">
@@ -1673,8 +1698,8 @@
           <t>Maintenance materials + contract maintenance</t>
         </is>
       </c>
-      <c r="B10" s="11">
-        <f>Inputs!$C$21</f>
+      <c r="B10" s="10">
+        <f>Inputs!$C$22</f>
         <v/>
       </c>
       <c r="C10" s="9" t="inlineStr">
@@ -1689,8 +1714,8 @@
           <t>Insurance (industrial)</t>
         </is>
       </c>
-      <c r="B11" s="11">
-        <f>Inputs!$C$22</f>
+      <c r="B11" s="10">
+        <f>Inputs!$C$23</f>
         <v/>
       </c>
       <c r="C11" s="9" t="inlineStr">
@@ -1705,8 +1730,8 @@
           <t>Contracted services (security/janitorial/IT/3rd-party MRV)</t>
         </is>
       </c>
-      <c r="B12" s="11">
-        <f>Inputs!$C$23</f>
+      <c r="B12" s="10">
+        <f>Inputs!$C$24</f>
         <v/>
       </c>
       <c r="C12" s="9" t="inlineStr">
@@ -1721,8 +1746,8 @@
           <t>G&amp;A / SG&amp;A</t>
         </is>
       </c>
-      <c r="B13" s="11">
-        <f>Inputs!$C$24</f>
+      <c r="B13" s="10">
+        <f>Inputs!$C$25</f>
         <v/>
       </c>
       <c r="C13" s="9" t="inlineStr">
@@ -1766,18 +1791,32 @@
     <row r="19">
       <c r="A19" s="12" t="inlineStr">
         <is>
-          <t>Labor ALONE (MI-adjusted)</t>
+          <t>Labor ALONE (MI-adj x cross-training)</t>
         </is>
       </c>
       <c r="B19" s="17">
-        <f>Inputs!$C$17*Inputs!$C$18</f>
+        <f>Inputs!$C$17*Inputs!$C$18*Inputs!$C$19</f>
         <v/>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="18" t="inlineStr">
         <is>
-          <t>-&gt; exceeds the signed model's entire implied opex above. Signed EBITDA overstates margin.</t>
+          <t>-&gt; at worst-case staffing, labor alone exceeds the signed model's entire implied opex. Signed EBITDA overstates margin.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="2" t="inlineStr">
+        <is>
+          <t>WasteWerx (V. Tizio, 5/27/26): staffing is intentional worst-case 'overkill'; cross-trained roles will reduce headcount;</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="2" t="inlineStr">
+        <is>
+          <t>health insurance &amp; benefits need actuals; salaries are FL market — Robert to adjust to Michigan pay rates. Flex via xtrain + mi_adj inputs.</t>
         </is>
       </c>
     </row>
@@ -1844,7 +1883,7 @@
           <t>Pyrolysis oil — raw, market price</t>
         </is>
       </c>
-      <c r="B5" s="10">
+      <c r="B5" s="11">
         <f>(Inputs!$C$5*Inputs!$C$6*Inputs!$C$7)*Inputs!$C$9</f>
         <v/>
       </c>
@@ -1865,7 +1904,7 @@
           <t>Carbon black</t>
         </is>
       </c>
-      <c r="B6" s="10">
+      <c r="B6" s="11">
         <f>(Inputs!$C$5*Inputs!$C$6*Inputs!$C$8)*Inputs!$C$10</f>
         <v/>
       </c>
@@ -1886,7 +1925,7 @@
           <t>Renewable diesel (upgraded fuel)</t>
         </is>
       </c>
-      <c r="B7" s="10">
+      <c r="B7" s="11">
         <f>Inputs!$C$11</f>
         <v/>
       </c>
@@ -1907,7 +1946,7 @@
           <t>SAF / kerosene (upgraded fuel)</t>
         </is>
       </c>
-      <c r="B8" s="10">
+      <c r="B8" s="11">
         <f>Inputs!$C$12</f>
         <v/>
       </c>
@@ -1928,7 +1967,7 @@
           <t>D4 RIN</t>
         </is>
       </c>
-      <c r="B9" s="11">
+      <c r="B9" s="10">
         <f>Inputs!$C$13</f>
         <v/>
       </c>
@@ -1949,7 +1988,7 @@
           <t>D7 RIN</t>
         </is>
       </c>
-      <c r="B10" s="11">
+      <c r="B10" s="10">
         <f>Inputs!$C$14</f>
         <v/>
       </c>
@@ -1970,7 +2009,7 @@
           <t>Section 45Z — RD</t>
         </is>
       </c>
-      <c r="B11" s="11">
+      <c r="B11" s="10">
         <f>Inputs!$C$15</f>
         <v/>
       </c>
@@ -1991,7 +2030,7 @@
           <t>Section 45Z — SAF</t>
         </is>
       </c>
-      <c r="B12" s="11">
+      <c r="B12" s="10">
         <f>Inputs!$C$16</f>
         <v/>
       </c>
@@ -2166,7 +2205,7 @@
         </is>
       </c>
       <c r="B24" s="15">
-        <f>Inputs!$C$25</f>
+        <f>Inputs!$C$26</f>
         <v/>
       </c>
     </row>
@@ -2177,7 +2216,7 @@
         </is>
       </c>
       <c r="B25" s="15">
-        <f>Inputs!$C$30+Inputs!$C$31+Inputs!$C$32+Inputs!$C$33</f>
+        <f>Inputs!$C$31+Inputs!$C$32+Inputs!$C$33+Inputs!$C$34</f>
         <v/>
       </c>
     </row>
@@ -2188,7 +2227,7 @@
         </is>
       </c>
       <c r="B26" s="15">
-        <f>Inputs!$C$34</f>
+        <f>Inputs!$C$35</f>
         <v/>
       </c>
     </row>
@@ -2228,7 +2267,7 @@
         </is>
       </c>
       <c r="B31" s="15">
-        <f>Inputs!$C$26+Inputs!$C$27+Inputs!$C$28+Inputs!$C$29</f>
+        <f>Inputs!$C$27+Inputs!$C$28+Inputs!$C$29+Inputs!$C$30</f>
         <v/>
       </c>
     </row>
@@ -2239,7 +2278,7 @@
         </is>
       </c>
       <c r="B32" s="23">
-        <f>Inputs!$C$25-B31</f>
+        <f>Inputs!$C$26-B31</f>
         <v/>
       </c>
       <c r="C32" s="2" t="inlineStr">
@@ -2321,7 +2360,7 @@
         <v/>
       </c>
       <c r="C5" s="19">
-        <f>Inputs!$C$36</f>
+        <f>Inputs!$C$37</f>
         <v/>
       </c>
       <c r="D5" s="21">
@@ -2345,7 +2384,7 @@
         <v/>
       </c>
       <c r="C6" s="19">
-        <f>Inputs!$C$36</f>
+        <f>Inputs!$C$37</f>
         <v/>
       </c>
       <c r="D6" s="21">
@@ -2369,7 +2408,7 @@
         <v/>
       </c>
       <c r="C7" s="19">
-        <f>Inputs!$C$36</f>
+        <f>Inputs!$C$37</f>
         <v/>
       </c>
       <c r="D7" s="22">
@@ -2393,7 +2432,7 @@
         <v/>
       </c>
       <c r="C8" s="19">
-        <f>Inputs!$C$36</f>
+        <f>Inputs!$C$37</f>
         <v/>
       </c>
       <c r="D8" s="22">
@@ -2417,7 +2456,7 @@
         <v/>
       </c>
       <c r="C9" s="19">
-        <f>Inputs!$C$36</f>
+        <f>Inputs!$C$37</f>
         <v/>
       </c>
       <c r="D9" s="22">
@@ -2441,7 +2480,7 @@
         <v/>
       </c>
       <c r="C10" s="19">
-        <f>Inputs!$C$36</f>
+        <f>Inputs!$C$37</f>
         <v/>
       </c>
       <c r="D10" s="21">
@@ -2465,7 +2504,7 @@
         <v/>
       </c>
       <c r="C11" s="19">
-        <f>Inputs!$C$36</f>
+        <f>Inputs!$C$37</f>
         <v/>
       </c>
       <c r="D11" s="21">
@@ -2535,7 +2574,7 @@
         </is>
       </c>
       <c r="B5" s="25">
-        <f>Inputs!$C$25</f>
+        <f>Inputs!$C$26</f>
         <v/>
       </c>
       <c r="C5" s="9" t="inlineStr">
@@ -2551,7 +2590,7 @@
         </is>
       </c>
       <c r="B6" s="25">
-        <f>Inputs!$C$25*Inputs!$C$36</f>
+        <f>Inputs!$C$26*Inputs!$C$37</f>
         <v/>
       </c>
       <c r="C6" s="9" t="inlineStr">
@@ -2567,7 +2606,7 @@
         </is>
       </c>
       <c r="B7" s="25">
-        <f>Inputs!$C$35</f>
+        <f>Inputs!$C$36</f>
         <v/>
       </c>
       <c r="C7" s="9" t="inlineStr">
@@ -2583,7 +2622,7 @@
         </is>
       </c>
       <c r="B8" s="25">
-        <f>Inputs!$C$25*Inputs!$C$36+Inputs!$C$35</f>
+        <f>Inputs!$C$26*Inputs!$C$37+Inputs!$C$36</f>
         <v/>
       </c>
       <c r="C8" s="9" t="inlineStr">
@@ -2603,7 +2642,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A31"/>
+  <dimension ref="A1:A33"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="116" customWidth="1" min="1" max="1"/>
@@ -2713,91 +2752,105 @@
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">    staffing pro forma and must be budgeted separately. Labor figure is FL market; add 5-10% for Michigan.</t>
+          <t xml:space="preserve">    staffing pro forma and must be budgeted separately. Labor is intentional WORST-CASE per WasteWerx (V. Tizio,</t>
         </is>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="2" t="inlineStr"/>
+      <c r="A18" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    5/27/26): cross-training reduces headcount (set xtrain&lt;1.0), salaries are FL market (set mi_adj for Michigan),</t>
+        </is>
+      </c>
     </row>
     <row r="19">
-      <c r="A19" s="3" t="inlineStr">
+      <c r="A19" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    and health-insurance/benefits actuals are still pending — net labor could move down (cross-training) or up (MI+benefits).</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="2" t="inlineStr"/>
+    </row>
+    <row r="21">
+      <c r="A21" s="3" t="inlineStr">
         <is>
           <t>CAPITAL</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  * Sponsor use-of-funds (~$16M) exceeds the $15M/site raise by ~$1M — confirm which line absorbs it.</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  * $2.5M company raise stays separate from site SPV totals.</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
+          <t xml:space="preserve">  * Sponsor use-of-funds (~$16M) exceeds the $15M/site raise by ~$1M — confirm which line absorbs it.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  * $2.5M company raise stays separate from site SPV totals.</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="2" t="inlineStr">
+        <is>
           <t xml:space="preserve">  * WasteWerx is a LICENSE, not a sale; title stays with WasteWerx; license fee depreciation differs; transfer/termination terms matter.</t>
         </is>
       </c>
     </row>
-    <row r="23">
-      <c r="A23" s="2" t="inlineStr"/>
-    </row>
-    <row r="24">
-      <c r="A24" s="3" t="inlineStr">
+    <row r="25">
+      <c r="A25" s="2" t="inlineStr"/>
+    </row>
+    <row r="26">
+      <c r="A26" s="3" t="inlineStr">
         <is>
           <t>GOVERNANCE / LEGAL</t>
-        </is>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  * Securities: not an offer; securities counsel review required before any circulation.</t>
-        </is>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  * PublicLogic = governance/document partner, NOT placement agent/broker-dealer; fee FIXED &amp; NON-CONTINGENT.</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">  * Community-benefit %: source files say 10%; sponsor flags a conflict — do not publish a number until reconciled.</t>
+          <t xml:space="preserve">  * Securities: not an offer; securities counsel review required before any circulation.</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">  * Final site list (Coldwater Phase 2 vs Lincoln) [CONFIRM]; parent-holdco legal name [CONFIRM].</t>
+          <t xml:space="preserve">  * PublicLogic = governance/document partner, NOT placement agent/broker-dealer; fee FIXED &amp; NON-CONTINGENT.</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">  * National Salvage: 'largest treated-wood recycler in the U.S.' unless stronger evidence (a verbal 'in the world' is unverified).</t>
+          <t xml:space="preserve">  * Community-benefit %: source files say 10%; sponsor flags a conflict — do not publish a number until reconciled.</t>
         </is>
       </c>
     </row>
     <row r="30">
-      <c r="A30" s="2" t="inlineStr"/>
+      <c r="A30" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  * Final site list (Coldwater Phase 2 vs Lincoln) [CONFIRM]; parent-holdco legal name [CONFIRM].</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  * National Salvage: 'largest treated-wood recycler in the U.S.' unless stronger evidence (a verbal 'in the world' is unverified).</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="2" t="inlineStr"/>
+    </row>
+    <row r="33">
+      <c r="A33" s="2" t="inlineStr">
         <is>
           <t>Not financial, accounting, securities, or tax advice. Figures trace to the canonical workbook / signed pro forma; verify before use.</t>
         </is>

</xml_diff>